<commit_message>
Historico_Cortes - siembra/append Sep-2026
</commit_message>
<xml_diff>
--- a/Tablas/Historico_Cortes.xlsx
+++ b/Tablas/Historico_Cortes.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1227,6 +1227,258 @@
       </c>
       <c r="J22" t="n">
         <v>8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>468</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-17</v>
+      </c>
+      <c r="E23" t="n">
+        <v>83</v>
+      </c>
+      <c r="F23" t="n">
+        <v>75</v>
+      </c>
+      <c r="G23" t="n">
+        <v>78</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="I23" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>131</v>
+      </c>
+      <c r="D24" t="n">
+        <v>66</v>
+      </c>
+      <c r="E24" t="n">
+        <v>56</v>
+      </c>
+      <c r="F24" t="n">
+        <v>81</v>
+      </c>
+      <c r="G24" t="n">
+        <v>10</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>3</v>
+      </c>
+      <c r="J24" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>470</v>
+      </c>
+      <c r="D25" t="n">
+        <v>21</v>
+      </c>
+      <c r="E25" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" t="n">
+        <v>28</v>
+      </c>
+      <c r="G25" t="n">
+        <v>57</v>
+      </c>
+      <c r="H25" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="I25" t="n">
+        <v>10</v>
+      </c>
+      <c r="J25" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>95</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-14</v>
+      </c>
+      <c r="E26" t="n">
+        <v>88</v>
+      </c>
+      <c r="F26" t="n">
+        <v>55</v>
+      </c>
+      <c r="G26" t="n">
+        <v>31</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>318</v>
+      </c>
+      <c r="D27" t="n">
+        <v>20</v>
+      </c>
+      <c r="E27" t="n">
+        <v>39</v>
+      </c>
+      <c r="F27" t="n">
+        <v>86</v>
+      </c>
+      <c r="G27" t="n">
+        <v>48</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2076</v>
+      </c>
+      <c r="D28" t="n">
+        <v>24</v>
+      </c>
+      <c r="E28" t="n">
+        <v>88</v>
+      </c>
+      <c r="F28" t="n">
+        <v>47</v>
+      </c>
+      <c r="G28" t="n">
+        <v>73</v>
+      </c>
+      <c r="H28" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="I28" t="n">
+        <v>6</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>515</v>
+      </c>
+      <c r="D29" t="n">
+        <v>13</v>
+      </c>
+      <c r="E29" t="n">
+        <v>72</v>
+      </c>
+      <c r="F29" t="n">
+        <v>59</v>
+      </c>
+      <c r="G29" t="n">
+        <v>73</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I29" t="n">
+        <v>4</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1240,7 +1492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E321"/>
+  <dimension ref="A1:E435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8413,6 +8665,2568 @@
         <v>1</v>
       </c>
     </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Luminaria superior e inferior apagada durante la noche</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>303</v>
+      </c>
+      <c r="E322" t="n">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Luminaria superior apagada durante la noche</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>58</v>
+      </c>
+      <c r="E323" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Luminaria inferior apagada durante la noche</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>33</v>
+      </c>
+      <c r="E324" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Columna en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>29</v>
+      </c>
+      <c r="E325" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Luminaria superior e inferior encendida de día</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>23</v>
+      </c>
+      <c r="E326" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Luminaria superior intermitente</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>11</v>
+      </c>
+      <c r="E327" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Tapa faltante/deteriorada</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>5</v>
+      </c>
+      <c r="E328" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Limpieza de luminaria</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>4</v>
+      </c>
+      <c r="E329" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>ALUMBRADO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Luminaria inferior intermitente</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Inconvenientes con intervenciones de arbolado</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>39</v>
+      </c>
+      <c r="E331" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Árbol obstruye luminaria</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>38</v>
+      </c>
+      <c r="E332" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Reparación de rejas, bancos, mesas y sillas en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>9</v>
+      </c>
+      <c r="E333" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Reparación de juegos/estaciones de ejercicio en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>9</v>
+      </c>
+      <c r="E334" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Reparación o daño de caniles en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D335" t="n">
+        <v>8</v>
+      </c>
+      <c r="E335" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Reparación de senderos en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>8</v>
+      </c>
+      <c r="E336" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Reparación de bebederos en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>6</v>
+      </c>
+      <c r="E337" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Árbol obstruye semáforo, cartel u otro elemento.</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>4</v>
+      </c>
+      <c r="E338" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Inconvenientes con las tareas de guardián de plaza</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>3</v>
+      </c>
+      <c r="E339" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Vaciado de cesto papelero en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>3</v>
+      </c>
+      <c r="E340" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Instalación de juegos en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>1</v>
+      </c>
+      <c r="E341" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Instalación de cestos de basura en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>1</v>
+      </c>
+      <c r="E342" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Inconvenientes con los horarios de apertura y cierre de parque/plaza</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>1</v>
+      </c>
+      <c r="E343" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>ARBOLADO Y PLAZAS</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Reposición de cesto papelero en parque/plaza</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>1</v>
+      </c>
+      <c r="E344" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Bache en calle de asfalto</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>166</v>
+      </c>
+      <c r="E345" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Reparación/construcción de cordón</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>111</v>
+      </c>
+      <c r="E346" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Bache en calle de hormigón</t>
+        </is>
+      </c>
+      <c r="D347" t="n">
+        <v>38</v>
+      </c>
+      <c r="E347" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Reparación de rampa de accesibilidad</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>36</v>
+      </c>
+      <c r="E348" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Construcción de cuneta</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Construcción de rampa de accesibilidad</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Repavimentación de calle</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Repintado / reparación de demarcación vial en calle o cordón</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>14</v>
+      </c>
+      <c r="E352" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Reparación de cuneta</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>13</v>
+      </c>
+      <c r="E353" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Inconvenientes con obras de bacheo</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>12</v>
+      </c>
+      <c r="E354" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Bache en calle de adoquines</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>8</v>
+      </c>
+      <c r="E355" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Reparación de vereda por obra mal terminada</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Reparación de lomo de burro o reductor de velocidad</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>4</v>
+      </c>
+      <c r="E357" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Refugio de colectivo en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Refugio de colectivo con riesgo de caída</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>2</v>
+      </c>
+      <c r="E359" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Reparación de rejas en esquina</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>2</v>
+      </c>
+      <c r="E360" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Reparación de calle por hundimiento/socavamiento</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>1</v>
+      </c>
+      <c r="E361" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Refugio de colectivo solicitud de limpieza</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>1</v>
+      </c>
+      <c r="E362" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Parada de colectivo (poste) en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>CALLES Y VEREDAS</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Reparación de tapa de empresa de servicio público en calle/vereda</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Otros ruidos molestos</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>29</v>
+      </c>
+      <c r="E365" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Falta de Habilitación - Actividad no declarada</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>19</v>
+      </c>
+      <c r="E366" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Presencia de plagas /roedores, cucarachas…etc)</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>12</v>
+      </c>
+      <c r="E367" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Derrame tóxico o material riesgoso</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>6</v>
+      </c>
+      <c r="E368" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Malos olores</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>5</v>
+      </c>
+      <c r="E369" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Obras fuera del horario permitido</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>4</v>
+      </c>
+      <c r="E370" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Actividad comercial fuera del horario habilitado</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>3</v>
+      </c>
+      <c r="E371" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Ruidos molestos por aires acondicionados</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Falta de higiene</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>2</v>
+      </c>
+      <c r="E373" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Venta de productos vencidos o en mal estado</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>2</v>
+      </c>
+      <c r="E374" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Música fuera del horario habilitado</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>2</v>
+      </c>
+      <c r="E375" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Venta de bebidas alcohólicas fuera del horario habilitado</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>2</v>
+      </c>
+      <c r="E376" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Venta no habilitada de bebidas alcohólicas</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>2</v>
+      </c>
+      <c r="E377" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Carga y descarga fuera del horario habilitado</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>2</v>
+      </c>
+      <c r="E378" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Ruidos Molestos por Autoelevadores</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>1</v>
+      </c>
+      <c r="E379" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>CONTROL DE ACTIVIDADES COMERCIALES</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Fumadores en espacios no permitidos</t>
+        </is>
+      </c>
+      <c r="D380" t="n">
+        <v>1</v>
+      </c>
+      <c r="E380" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Cable cortado</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>117</v>
+      </c>
+      <c r="E381" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Roedores en espacio público</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>83</v>
+      </c>
+      <c r="E382" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Reparación de vereda rota por empresa de servicio</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>27</v>
+      </c>
+      <c r="E383" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Poste en mal estado/sin mantenimiento</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>21</v>
+      </c>
+      <c r="E384" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Agua servida en la vía pública proveniente de comercio o industria</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>14</v>
+      </c>
+      <c r="E385" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Ocupación irregular de objetos y/o vehículos</t>
+        </is>
+      </c>
+      <c r="D386" t="n">
+        <v>8</v>
+      </c>
+      <c r="E386" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Abejas en espacio público</t>
+        </is>
+      </c>
+      <c r="D387" t="n">
+        <v>7</v>
+      </c>
+      <c r="E387" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Desobstrucción de cloacas</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>7</v>
+      </c>
+      <c r="E388" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Eventos irregulares en vía pública</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Retiro de afiches y/o pasacalles</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>4</v>
+      </c>
+      <c r="E390" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Inconvenientes con el suministro de agua</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>4</v>
+      </c>
+      <c r="E391" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Garita/puestos de diarios y/o flores irregulares</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>3</v>
+      </c>
+      <c r="E392" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Poste quebrado/cortado</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>3</v>
+      </c>
+      <c r="E393" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Incon. En cámaras de inspec. de empresa de servicio público en calle/vereda</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>2</v>
+      </c>
+      <c r="E394" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Marquesinas/Carteles en locales comerciales</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>2</v>
+      </c>
+      <c r="E395" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Hidrolavado por grafitis/pegatinas</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>2</v>
+      </c>
+      <c r="E396" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Olores nauseabundos en vía pública</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Toldos/cerramientos/estructuras irregulares en vía pública</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>2</v>
+      </c>
+      <c r="E398" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Reparación de calle rota por empresa de servicio</t>
+        </is>
+      </c>
+      <c r="D399" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Mosquitos en espacio público</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>1</v>
+      </c>
+      <c r="E400" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Otras plagas en espacio público</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Nivelación de tapa de empresa de servicio público en calle/vereda</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>CONTROL DEL ESPACIO PUBLICO</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Avispas en espacio público</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Retiro de escombros y/o restos de obra</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>605</v>
+      </c>
+      <c r="E404" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Retiro de restos de poda y/o jardinería domiciliaria</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>423</v>
+      </c>
+      <c r="E405" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Retiro de objetos/elementos en desuso</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>243</v>
+      </c>
+      <c r="E406" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Retiro de muebles y/o electrodomésticos en desuso</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>181</v>
+      </c>
+      <c r="E407" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Falta de barrido o barrido deficiente</t>
+        </is>
+      </c>
+      <c r="D408" t="n">
+        <v>179</v>
+      </c>
+      <c r="E408" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Falta de recolección de residuos orgánicos/húmedos</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>120</v>
+      </c>
+      <c r="E409" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Limpieza/higienización de espacio público</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>77</v>
+      </c>
+      <c r="E410" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Falta de recolección de residuos reciclables (Programa Día Verde)</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>51</v>
+      </c>
+      <c r="E411" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Retiro de restos de poda y/o de arbolado público</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>42</v>
+      </c>
+      <c r="E412" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Yuyos/malezas/césped no cortado/plantas que interfieren en vía pública</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>40</v>
+      </c>
+      <c r="E413" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Vaciado de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>35</v>
+      </c>
+      <c r="E414" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Yuyos/malezas/césped no cortado/plantas</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>16</v>
+      </c>
+      <c r="E415" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Colocación de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>11</v>
+      </c>
+      <c r="E416" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Vaciado de contenedor</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>10</v>
+      </c>
+      <c r="E417" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Reposición de contenedor</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>7</v>
+      </c>
+      <c r="E418" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Personal de empresa de recolección con conductas indebidas</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Retiro de animales muertos en vía pública</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>7</v>
+      </c>
+      <c r="E420" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Reposición de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>7</v>
+      </c>
+      <c r="E421" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Irregularidades en la disposición de residuos húmedos/orgánicos</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>5</v>
+      </c>
+      <c r="E422" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Reparación de cesto papelero</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>4</v>
+      </c>
+      <c r="E423" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Acopio de cartoneros en espacio público</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Personal de empresa de recolección realiza pedido de dádivas</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>1</v>
+      </c>
+      <c r="E425" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Lavado de contenedor</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>1</v>
+      </c>
+      <c r="E426" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>RESIDUOS Y LIMPIEZA</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Camión de recolección que incumple normas de tránsito</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Vehículos Abandonados</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>392</v>
+      </c>
+      <c r="E428" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Reparación de semáforo</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>77</v>
+      </c>
+      <c r="E429" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Vehículo mal estacionado</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>15</v>
+      </c>
+      <c r="E430" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Reparación de señal de tránsito</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>9</v>
+      </c>
+      <c r="E431" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Remoción de volquete abandonado o mal dispuesto</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>7</v>
+      </c>
+      <c r="E432" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Instalación de cartel nomenclador de calle</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Reparación de cartel nomenclador de calle</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>5</v>
+      </c>
+      <c r="E434" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>TRANSITO</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Vehículo obstruyendo garage</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>